<commit_message>
Update spark logbook (1 entries) — 2026-08-04T01:15:56.929Z
</commit_message>
<xml_diff>
--- a/spark-logbook.xlsx
+++ b/spark-logbook.xlsx
@@ -428,13 +428,13 @@
         <v>2026-08-04</v>
       </c>
       <c r="B2" t="str">
-        <v>09:00</v>
+        <v>08:13</v>
       </c>
       <c r="C2" t="str">
         <v>Service</v>
       </c>
       <c r="D2" t="str">
-        <v>Replaced west spark detector on zone 5 (dust collector) due To false alarms</v>
+        <v>Replaced West Spark Detector due to False alarms</v>
       </c>
       <c r="E2" t="str">
         <v>Tim Rohner</v>

</xml_diff>